<commit_message>
kill added for current user
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55646C\Documents\GitHub\P003_090_TimesheetApprovals_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3707280C-B28B-4631-966E-6ED1F53446D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FCE976-BC50-47A7-ADE3-F0AF2DC8C1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
filter hire date was added in no time reported
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55646C\Documents\GitHub\P003_090_TimesheetApprovals_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FCE976-BC50-47A7-ADE3-F0AF2DC8C1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF16036-9F53-4C56-B9E0-63D82BE09E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
Updated to allow for multiple agencies
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55646C\Documents\GitHub\P003_090_TimesheetApprovals_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\57145C\Documents\UiPath\P003_090_TimesheetApprovals_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF16036-9F53-4C56-B9E0-63D82BE09E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16ADBD81-D6EF-45B7-A6FC-EA5D55CF22A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -199,479 +199,479 @@
     <t>Sheet1</t>
   </si>
   <si>
+    <t>Missing time Count</t>
+  </si>
+  <si>
+    <t>NotSubmittedSummaryReportFileName</t>
+  </si>
+  <si>
+    <t>NotSubmitteSummaryReportSheetName</t>
+  </si>
+  <si>
+    <t>NotSubmittedSummaryReportTemplatePath</t>
+  </si>
+  <si>
+    <t>NotApprovedSummaryReportFileName</t>
+  </si>
+  <si>
+    <t>NotApprovedSummaryReportSheetName</t>
+  </si>
+  <si>
+    <t>NotApprovedSummaryReportTemplatePath</t>
+  </si>
+  <si>
+    <t>EmpIDHeaderInNotSubmittedWeeklyReport</t>
+  </si>
+  <si>
+    <t>HeaderRowNoInNotSubmittedSummaryReport</t>
+  </si>
+  <si>
+    <t>EmpIDHeaderInNotSubmittedSummaryReport</t>
+  </si>
+  <si>
+    <t>TimeSheet Entry / Approval Reminders Automation – Time Not Submitted/Incomplete - Monthly Summary Report – {month}{year}</t>
+  </si>
+  <si>
+    <t>HeaderRowNoInNotApprovedSummaryReport</t>
+  </si>
+  <si>
+    <t>CounterHeaderInNotApprovedSummaryReport</t>
+  </si>
+  <si>
+    <t>CounterHeaderInNotSubmittedSummaryReport</t>
+  </si>
+  <si>
+    <t>Not Approved Count</t>
+  </si>
+  <si>
+    <t>TimeSheet Entry / Approval Reminders Automation – Time Not Approved - Monthly Summary Report – {month}{year}</t>
+  </si>
+  <si>
+    <t>Incomplete time Count</t>
+  </si>
+  <si>
+    <t>EmpTypeHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>ManagementLevelHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>Management Level</t>
+  </si>
+  <si>
+    <t>EmpTypeFilterValueInRPT00177</t>
+  </si>
+  <si>
+    <t>ManagementLevelFilterValueInRPT00177</t>
+  </si>
+  <si>
+    <t>Board Member</t>
+  </si>
+  <si>
+    <t>NoTimeReportedFileName</t>
+  </si>
+  <si>
+    <t>EmailheaderInRPT00177</t>
+  </si>
+  <si>
+    <t>ManagerEmailHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>NoTimeReportedMailSubject</t>
+  </si>
+  <si>
+    <t>No Time Reported – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
+  </si>
+  <si>
+    <t>StatusHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>StatusFilterValueForNotSubmitted</t>
+  </si>
+  <si>
+    <t>Not Submitted</t>
+  </si>
+  <si>
+    <t>NotSubmittedFileName</t>
+  </si>
+  <si>
+    <t>ManagerEmailHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>EmailheaderInRPT00169</t>
+  </si>
+  <si>
+    <t>StatusFilterValueForNotApproved</t>
+  </si>
+  <si>
+    <t>Submitted</t>
+  </si>
+  <si>
+    <t>NotSubmittedMailSubject</t>
+  </si>
+  <si>
+    <t>NotApprovedMailSubject</t>
+  </si>
+  <si>
+    <t>WorkerHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>Worker</t>
+  </si>
+  <si>
+    <t>ManagerHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>LocationHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>WorkerHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>ManagerHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>LocationHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>MangerIDHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>EmpIDHeaderInNotApprovedWeeklyReport</t>
+  </si>
+  <si>
+    <t>EmpIDHeaderInNotApprovedSummaryReport</t>
+  </si>
+  <si>
+    <t>NoTimeReportedSummaryMailSubject</t>
+  </si>
+  <si>
+    <t>NotSubmittedSummaryMailSubject</t>
+  </si>
+  <si>
+    <t>NotApprovedSummaryMailSubject</t>
+  </si>
+  <si>
+    <t>ExMailSubject</t>
+  </si>
+  <si>
+    <t>NotApprovedFileName</t>
+  </si>
+  <si>
+    <t>Time Not Approved - WK{week} - {month} - {datetime}.xlsx</t>
+  </si>
+  <si>
+    <t>WorkerTypeFilterValueInRPT00177</t>
+  </si>
+  <si>
+    <t>WorkerTypeHeaderInRPT00177</t>
+  </si>
+  <si>
+    <t>primaryWorkEmail</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_PayCycleWeekMondayDate</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SummaryMailTime</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_MailAccount</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_ExceptionToMail</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_ExceptionCcMail</t>
+  </si>
+  <si>
+    <t>O365TenantIDAssetName</t>
+  </si>
+  <si>
+    <t>Shared_O365TenantID</t>
+  </si>
+  <si>
+    <t>O365ApplicationIDAssetName</t>
+  </si>
+  <si>
+    <t>Shared_O365ApplicationID</t>
+  </si>
+  <si>
+    <t>O365ApplicationSecretAssetName</t>
+  </si>
+  <si>
+    <t>Shared_O365ApplicationSecret</t>
+  </si>
+  <si>
+    <t>O365AssetsInOrchestratorFolder</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_Queue</t>
+  </si>
+  <si>
+    <t>Time Not Approved – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
+  </si>
+  <si>
+    <t>LocalDownloadPath</t>
+  </si>
+  <si>
+    <t>Sample_No time Reported_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
+  </si>
+  <si>
+    <t>Sample_Not Approved_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
+  </si>
+  <si>
+    <t>Sample_Not Submitted_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
+  </si>
+  <si>
+    <t>Regular</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_WeeklyEmailCC</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_WeeklyEmailTO</t>
+  </si>
+  <si>
+    <t>Monthly summary report - No Time Reported - {currentMonth} {year}.xlsx</t>
+  </si>
+  <si>
+    <t>TimeSheet Entry / Approval Reminders Automation –No Time Reported - Monthly Summary Report – {month} {year}</t>
+  </si>
+  <si>
+    <t>Monthly summary report - Not Submitted - {currentMonth} {year}.xlsx</t>
+  </si>
+  <si>
+    <t>Monthly summary report - Not Approved - {currentMonth} {year}.xlsx</t>
+  </si>
+  <si>
+    <t>Time Not submitted - WK{week} - {month} - {datetime}.xlsx</t>
+  </si>
+  <si>
+    <t>Time Not Submitted – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
+  </si>
+  <si>
+    <t>SE_SPUnavailable</t>
+  </si>
+  <si>
+    <t>Bot was not able to access the Sharepoint at this time due to connectivity issues.</t>
+  </si>
+  <si>
+    <t>BE_InvalidReqType</t>
+  </si>
+  <si>
+    <t>Bot was not able to process the request since it was not defined.</t>
+  </si>
+  <si>
+    <t>SE_FileNotFound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bot was not able to find the file at the provided location </t>
+  </si>
+  <si>
+    <t>Timeout</t>
+  </si>
+  <si>
+    <t>SharepointInputFolderName</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>SharepointOutputFolderName</t>
+  </si>
+  <si>
+    <t>00:01:00</t>
+  </si>
+  <si>
+    <t>No Time Reported - WK{week} - {month} - {datetime}.xlsx</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SummaryMailTo</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SummaryMailCC</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SPURL</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SPRootFolder</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_SummaryFolder</t>
+  </si>
+  <si>
+    <t>BotAutomationFolder</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>BotWorkingFolder</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_LocalRootFolder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System Exception - </t>
+  </si>
+  <si>
+    <t>C:\</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals</t>
+  </si>
+  <si>
+    <t>SendEmailSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send email workflow has system exception </t>
+  </si>
+  <si>
+    <t>SaveFileSPSE</t>
+  </si>
+  <si>
+    <t>Save file into sharepoint workflow has system exception</t>
+  </si>
+  <si>
+    <t>CreateFoldersSPSE</t>
+  </si>
+  <si>
+    <t>Create folders into sharepoint has system exception</t>
+  </si>
+  <si>
+    <t>CreateSummaryReportSE</t>
+  </si>
+  <si>
+    <t>Check and create summary report workflow has system exception</t>
+  </si>
+  <si>
+    <t>GenerateSummaryReportSE</t>
+  </si>
+  <si>
+    <t>Generate summary report workflow has system exception</t>
+  </si>
+  <si>
+    <t>NotApprovedReportSE</t>
+  </si>
+  <si>
+    <t>NotSubmittedReportSE</t>
+  </si>
+  <si>
+    <t>NoTimeReportedReportSE</t>
+  </si>
+  <si>
+    <t>Not Approved monthly summary report workflow has system exception</t>
+  </si>
+  <si>
+    <t>Not Submitted monthly summary report workflow has system exception</t>
+  </si>
+  <si>
+    <t>No Time Reported monthly summary report workflow has system exception</t>
+  </si>
+  <si>
+    <t>WeeklyNoTimeReportSE</t>
+  </si>
+  <si>
+    <t>WeeklyNotSubmittedSE</t>
+  </si>
+  <si>
+    <t>WeeklyNotApprovedSE</t>
+  </si>
+  <si>
+    <t>No Time Reported weekly report has system exception</t>
+  </si>
+  <si>
+    <t>Not Submitted weekly report has system exception</t>
+  </si>
+  <si>
+    <t>Not Approved weekly report has system exception</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NoTimeReportedSummaryMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NotSubmittedSummaryMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NotApprovedSummaryMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NoTimeReportedMailBody_PayCycleWeek</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NoTimeReportedMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NotApprovedMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_NotSubmittedMailBody</t>
+  </si>
+  <si>
+    <t>P003_090_TimesheetApprovals_ExceptionMailBody</t>
+  </si>
+  <si>
+    <t>AwaitingEmailHeaderInRPT00169</t>
+  </si>
+  <si>
+    <t>HireDateHeaderIn177</t>
+  </si>
+  <si>
+    <t>BotEnvironmentFolder</t>
+  </si>
+  <si>
+    <t>CF_-_Awaiting_Persons_Emails_PT</t>
+  </si>
+  <si>
+    <t>PROD</t>
+  </si>
+  <si>
+    <t>EmployeeType</t>
+  </si>
+  <si>
+    <t>ManagerEmail</t>
+  </si>
+  <si>
+    <t>PrimaryWorkEmail</t>
+  </si>
+  <si>
+    <t>WorkerType</t>
+  </si>
+  <si>
+    <t>HireDate</t>
+  </si>
+  <si>
+    <t>ManagerID</t>
+  </si>
+  <si>
+    <t>ReportedStatus</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
     <t>Emp ID</t>
-  </si>
-  <si>
-    <t>Missing time Count</t>
-  </si>
-  <si>
-    <t>NotSubmittedSummaryReportFileName</t>
-  </si>
-  <si>
-    <t>NotSubmitteSummaryReportSheetName</t>
-  </si>
-  <si>
-    <t>NotSubmittedSummaryReportTemplatePath</t>
-  </si>
-  <si>
-    <t>NotApprovedSummaryReportFileName</t>
-  </si>
-  <si>
-    <t>NotApprovedSummaryReportSheetName</t>
-  </si>
-  <si>
-    <t>NotApprovedSummaryReportTemplatePath</t>
-  </si>
-  <si>
-    <t>EmpIDHeaderInNotSubmittedWeeklyReport</t>
-  </si>
-  <si>
-    <t>HeaderRowNoInNotSubmittedSummaryReport</t>
-  </si>
-  <si>
-    <t>EmpIDHeaderInNotSubmittedSummaryReport</t>
-  </si>
-  <si>
-    <t>TimeSheet Entry / Approval Reminders Automation – Time Not Submitted/Incomplete - Monthly Summary Report – {month}{year}</t>
-  </si>
-  <si>
-    <t>HeaderRowNoInNotApprovedSummaryReport</t>
-  </si>
-  <si>
-    <t>CounterHeaderInNotApprovedSummaryReport</t>
-  </si>
-  <si>
-    <t>CounterHeaderInNotSubmittedSummaryReport</t>
-  </si>
-  <si>
-    <t>Not Approved Count</t>
-  </si>
-  <si>
-    <t>TimeSheet Entry / Approval Reminders Automation – Time Not Approved - Monthly Summary Report – {month}{year}</t>
-  </si>
-  <si>
-    <t>Incomplete time Count</t>
-  </si>
-  <si>
-    <t>EmpTypeHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>ManagementLevelHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>Management Level</t>
-  </si>
-  <si>
-    <t>EmpTypeFilterValueInRPT00177</t>
-  </si>
-  <si>
-    <t>ManagementLevelFilterValueInRPT00177</t>
-  </si>
-  <si>
-    <t>Board Member</t>
-  </si>
-  <si>
-    <t>NoTimeReportedFileName</t>
-  </si>
-  <si>
-    <t>EmailheaderInRPT00177</t>
-  </si>
-  <si>
-    <t>ManagerEmailHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>NoTimeReportedMailSubject</t>
-  </si>
-  <si>
-    <t>No Time Reported – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
-  </si>
-  <si>
-    <t>StatusHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>StatusFilterValueForNotSubmitted</t>
-  </si>
-  <si>
-    <t>Not Submitted</t>
-  </si>
-  <si>
-    <t>NotSubmittedFileName</t>
-  </si>
-  <si>
-    <t>ManagerEmailHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>EmailheaderInRPT00169</t>
-  </si>
-  <si>
-    <t>StatusFilterValueForNotApproved</t>
-  </si>
-  <si>
-    <t>Submitted</t>
-  </si>
-  <si>
-    <t>NotSubmittedMailSubject</t>
-  </si>
-  <si>
-    <t>NotApprovedMailSubject</t>
-  </si>
-  <si>
-    <t>WorkerHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>Worker</t>
-  </si>
-  <si>
-    <t>ManagerHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>LocationHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>WorkerHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>ManagerHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>Manager</t>
-  </si>
-  <si>
-    <t>LocationHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>MangerIDHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>EmpIDHeaderInNotApprovedWeeklyReport</t>
-  </si>
-  <si>
-    <t>EmpIDHeaderInNotApprovedSummaryReport</t>
-  </si>
-  <si>
-    <t>NoTimeReportedSummaryMailSubject</t>
-  </si>
-  <si>
-    <t>NotSubmittedSummaryMailSubject</t>
-  </si>
-  <si>
-    <t>NotApprovedSummaryMailSubject</t>
-  </si>
-  <si>
-    <t>ExMailSubject</t>
-  </si>
-  <si>
-    <t>NotApprovedFileName</t>
-  </si>
-  <si>
-    <t>Time Not Approved - WK{week} - {month} - {datetime}.xlsx</t>
-  </si>
-  <si>
-    <t>WorkerTypeFilterValueInRPT00177</t>
-  </si>
-  <si>
-    <t>WorkerTypeHeaderInRPT00177</t>
-  </si>
-  <si>
-    <t>Employee_ID</t>
-  </si>
-  <si>
-    <t>primaryWorkEmail</t>
-  </si>
-  <si>
-    <t>Manager_Email</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>Employee_Type</t>
-  </si>
-  <si>
-    <t>Reported_Status</t>
-  </si>
-  <si>
-    <t>Manager_ID</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_PayCycleWeekMondayDate</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SummaryMailTime</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_MailAccount</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_ExceptionToMail</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_ExceptionCcMail</t>
-  </si>
-  <si>
-    <t>O365TenantIDAssetName</t>
-  </si>
-  <si>
-    <t>Shared_O365TenantID</t>
-  </si>
-  <si>
-    <t>O365ApplicationIDAssetName</t>
-  </si>
-  <si>
-    <t>Shared_O365ApplicationID</t>
-  </si>
-  <si>
-    <t>O365ApplicationSecretAssetName</t>
-  </si>
-  <si>
-    <t>Shared_O365ApplicationSecret</t>
-  </si>
-  <si>
-    <t>O365AssetsInOrchestratorFolder</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_Queue</t>
-  </si>
-  <si>
-    <t>Time Not Approved – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
-  </si>
-  <si>
-    <t>Worker_Type</t>
-  </si>
-  <si>
-    <t>LocalDownloadPath</t>
-  </si>
-  <si>
-    <t>Sample_No time Reported_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
-  </si>
-  <si>
-    <t>Sample_Not Approved_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
-  </si>
-  <si>
-    <t>Sample_Not Submitted_Monthly Summary Report_TimeSheet Reminder.xlsx</t>
-  </si>
-  <si>
-    <t>Regular</t>
-  </si>
-  <si>
-    <t>Employee</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_WeeklyEmailCC</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_WeeklyEmailTO</t>
-  </si>
-  <si>
-    <t>Monthly summary report - No Time Reported - {currentMonth} {year}.xlsx</t>
-  </si>
-  <si>
-    <t>TimeSheet Entry / Approval Reminders Automation –No Time Reported - Monthly Summary Report – {month} {year}</t>
-  </si>
-  <si>
-    <t>Monthly summary report - Not Submitted - {currentMonth} {year}.xlsx</t>
-  </si>
-  <si>
-    <t>Monthly summary report - Not Approved - {currentMonth} {year}.xlsx</t>
-  </si>
-  <si>
-    <t>Time Not submitted - WK{week} - {month} - {datetime}.xlsx</t>
-  </si>
-  <si>
-    <t>Time Not Submitted – Week {week} {startmonth} {startday} – {endmonth} {endday}</t>
-  </si>
-  <si>
-    <t>SE_SPUnavailable</t>
-  </si>
-  <si>
-    <t>Bot was not able to access the Sharepoint at this time due to connectivity issues.</t>
-  </si>
-  <si>
-    <t>BE_InvalidReqType</t>
-  </si>
-  <si>
-    <t>Bot was not able to process the request since it was not defined.</t>
-  </si>
-  <si>
-    <t>SE_FileNotFound</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bot was not able to find the file at the provided location </t>
-  </si>
-  <si>
-    <t>Timeout</t>
-  </si>
-  <si>
-    <t>SharepointInputFolderName</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>Output</t>
-  </si>
-  <si>
-    <t>SharepointOutputFolderName</t>
-  </si>
-  <si>
-    <t>00:01:00</t>
-  </si>
-  <si>
-    <t>No Time Reported - WK{week} - {month} - {datetime}.xlsx</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SummaryMailTo</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SummaryMailCC</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SPURL</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SPRootFolder</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_SummaryFolder</t>
-  </si>
-  <si>
-    <t>BotAutomationFolder</t>
-  </si>
-  <si>
-    <t>Automation</t>
-  </si>
-  <si>
-    <t>BotWorkingFolder</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_LocalRootFolder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System Exception - </t>
-  </si>
-  <si>
-    <t>C:\</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals</t>
-  </si>
-  <si>
-    <t>SendEmailSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Send email workflow has system exception </t>
-  </si>
-  <si>
-    <t>SaveFileSPSE</t>
-  </si>
-  <si>
-    <t>Save file into sharepoint workflow has system exception</t>
-  </si>
-  <si>
-    <t>CreateFoldersSPSE</t>
-  </si>
-  <si>
-    <t>Create folders into sharepoint has system exception</t>
-  </si>
-  <si>
-    <t>CreateSummaryReportSE</t>
-  </si>
-  <si>
-    <t>Check and create summary report workflow has system exception</t>
-  </si>
-  <si>
-    <t>GenerateSummaryReportSE</t>
-  </si>
-  <si>
-    <t>Generate summary report workflow has system exception</t>
-  </si>
-  <si>
-    <t>NotApprovedReportSE</t>
-  </si>
-  <si>
-    <t>NotSubmittedReportSE</t>
-  </si>
-  <si>
-    <t>NoTimeReportedReportSE</t>
-  </si>
-  <si>
-    <t>Not Approved monthly summary report workflow has system exception</t>
-  </si>
-  <si>
-    <t>Not Submitted monthly summary report workflow has system exception</t>
-  </si>
-  <si>
-    <t>No Time Reported monthly summary report workflow has system exception</t>
-  </si>
-  <si>
-    <t>WeeklyNoTimeReportSE</t>
-  </si>
-  <si>
-    <t>WeeklyNotSubmittedSE</t>
-  </si>
-  <si>
-    <t>WeeklyNotApprovedSE</t>
-  </si>
-  <si>
-    <t>No Time Reported weekly report has system exception</t>
-  </si>
-  <si>
-    <t>Not Submitted weekly report has system exception</t>
-  </si>
-  <si>
-    <t>Not Approved weekly report has system exception</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NoTimeReportedSummaryMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NotSubmittedSummaryMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NotApprovedSummaryMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NoTimeReportedMailBody_PayCycleWeek</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NoTimeReportedMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NotApprovedMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_NotSubmittedMailBody</t>
-  </si>
-  <si>
-    <t>P003_090_TimesheetApprovals_ExceptionMailBody</t>
-  </si>
-  <si>
-    <t>AwaitingEmailHeaderInRPT00169</t>
-  </si>
-  <si>
-    <t>Hire_Date</t>
-  </si>
-  <si>
-    <t>HireDateHeaderIn177</t>
-  </si>
-  <si>
-    <t>BotEnvironmentFolder</t>
-  </si>
-  <si>
-    <t>CF_-_Awaiting_Persons_Emails_PT</t>
-  </si>
-  <si>
-    <t>PROD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -709,6 +709,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF444444"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -731,7 +737,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -744,6 +750,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1060,12 +1067,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z1006"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="155.28515625" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="47.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="155.26953125" customWidth="1"/>
+    <col min="3" max="3" width="81.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1107,13 +1114,13 @@
         <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.5">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -1126,7 +1133,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="29">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1144,7 +1151,7 @@
         <v>44</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
@@ -1160,7 +1167,7 @@
         <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -1168,7 +1175,7 @@
         <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
@@ -1176,7 +1183,7 @@
         <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -1184,7 +1191,7 @@
         <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
@@ -1197,24 +1204,24 @@
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>52</v>
@@ -1222,31 +1229,31 @@
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>112</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -1254,32 +1261,32 @@
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>52</v>
@@ -1287,23 +1294,23 @@
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B30" t="s">
         <v>48</v>
@@ -1311,7 +1318,7 @@
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31">
         <v>3</v>
@@ -1319,264 +1326,264 @@
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B35" t="s">
         <v>92</v>
-      </c>
-      <c r="B35" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" t="s">
-        <v>113</v>
+        <v>77</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>114</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B39" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B40" t="s">
-        <v>116</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" t="s">
         <v>72</v>
-      </c>
-      <c r="B41" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" t="s">
         <v>75</v>
-      </c>
-      <c r="B43" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>79</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" t="s">
         <v>98</v>
-      </c>
-      <c r="B48" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" t="s">
-        <v>114</v>
+        <v>201</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>118</v>
+        <v>205</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B52" t="s">
-        <v>117</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
+        <v>82</v>
+      </c>
+      <c r="B53" t="s">
         <v>83</v>
-      </c>
-      <c r="B53" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B54" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="14.5">
       <c r="A56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" t="s">
         <v>88</v>
-      </c>
-      <c r="B56" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.25" customHeight="1">
       <c r="A58" t="s">
+        <v>107</v>
+      </c>
+      <c r="B58" t="s">
         <v>108</v>
-      </c>
-      <c r="B58" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1">
       <c r="A61" t="s">
-        <v>111</v>
-      </c>
-      <c r="B61" t="s">
-        <v>133</v>
+        <v>110</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.25" customHeight="1">
       <c r="A62" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B62" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.25" customHeight="1">
       <c r="A63" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B63" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.25" customHeight="1">
       <c r="A64" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B64" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="14.25" customHeight="1">
       <c r="A65" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B65" t="str">
         <f>Constants!B2</f>
@@ -1585,175 +1592,175 @@
     </row>
     <row r="66" spans="1:2" ht="14.25" customHeight="1">
       <c r="A66" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B66" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.25" customHeight="1">
       <c r="A67" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="B67" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="14.25" customHeight="1">
       <c r="A68" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B68" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.25" customHeight="1">
       <c r="A69" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="B69" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.25" customHeight="1">
       <c r="A70" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.25" customHeight="1">
       <c r="A71" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B71" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.25" customHeight="1">
       <c r="A72" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B72" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.25" customHeight="1">
       <c r="A73" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B73" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.25" customHeight="1">
       <c r="A74" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="B74" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.25" customHeight="1">
       <c r="A75" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B75" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.25" customHeight="1">
       <c r="A76" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="B76" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="14.25" customHeight="1">
       <c r="A77" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B77" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="14.25" customHeight="1">
       <c r="A78" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B78" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="14.25" customHeight="1">
       <c r="A79" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="B79" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="14.25" customHeight="1">
       <c r="A80" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="B80" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="14.25" customHeight="1">
       <c r="A81" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B81" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="14.25" customHeight="1">
       <c r="A82" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B82" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="14.25" customHeight="1">
       <c r="A83" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B83" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="14.25" customHeight="1">
       <c r="A84" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B84" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="14.25" customHeight="1">
       <c r="A85" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B85" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="14.25" customHeight="1">
       <c r="A86" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="14.25" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>204</v>
@@ -2688,12 +2695,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z989"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2732,10 +2739,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2762,7 +2769,7 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="30">
+    <row r="3" spans="1:26" ht="29">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2773,7 +2780,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="45">
+    <row r="4" spans="1:26" ht="43.5">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -2887,7 +2894,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="18" spans="1:3" ht="45">
+    <row r="18" spans="1:3" ht="29">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -3878,12 +3885,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z982"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="86.28515625" customWidth="1"/>
-    <col min="2" max="2" width="53.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="86.26953125" customWidth="1"/>
+    <col min="2" max="2" width="53.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.26953125" customWidth="1"/>
+    <col min="4" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3924,10 +3931,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C2" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3936,10 +3943,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C3" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3949,10 +3956,10 @@
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C4" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3962,10 +3969,10 @@
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C5" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3974,10 +3981,10 @@
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C6" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3986,10 +3993,10 @@
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C7" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -3998,10 +4005,10 @@
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="B8" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C8" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4010,10 +4017,10 @@
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C9" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4023,10 +4030,10 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C10" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4035,10 +4042,10 @@
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="B11" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C11" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4047,10 +4054,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B12" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C12" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4059,10 +4066,10 @@
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B13" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C13" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4071,10 +4078,10 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B14" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C14" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4083,10 +4090,10 @@
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B15" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C15" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4095,10 +4102,10 @@
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C16" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4107,10 +4114,10 @@
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C17" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4119,10 +4126,10 @@
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C18" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4131,10 +4138,10 @@
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C19" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4143,10 +4150,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B20" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C20" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4155,10 +4162,10 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B21" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C21" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>
@@ -4167,10 +4174,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B22" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C22" t="str">
         <f>_xlfn.CONCAT(Constants!B2,"/P003_090_TimesheetApprovals")</f>

</xml_diff>